<commit_message>
Add metric script, license and paper PDF
- evaluation/runners/pilot_metrics.py computes every number in the paper
  from the stored logs and compares it with the stored tables; the main-flow
  metrics were previously computed by one-off commands that were not saved
- results/paper_numbers.csv lists each number with its denominator and source
- Rebuild the stale summaries that still showed 45 text-only answers
- Correct P047 precision@10 (0.1 to 0.111); reported mean and SD unchanged
- README: how each metric is computed, known paper count discrepancy
- Add MIT license and the paper PDF

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research_evaluation_20261030/results/recall_precision.xlsx
+++ b/research_evaluation_20261030/results/recall_precision.xlsx
@@ -519,55 +519,55 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C2" t="n">
-        <v>0.919</v>
+        <v>0.905</v>
       </c>
       <c r="D2" t="n">
-        <v>0.221</v>
+        <v>0.222</v>
       </c>
       <c r="E2" t="n">
-        <v>0.12</v>
+        <v>0.126</v>
       </c>
       <c r="F2" t="n">
-        <v>0.055</v>
+        <v>0.06</v>
       </c>
       <c r="G2" t="n">
-        <v>0.956</v>
+        <v>0.955</v>
       </c>
       <c r="H2" t="n">
-        <v>0.179</v>
+        <v>0.173</v>
       </c>
       <c r="I2" t="n">
-        <v>0.956</v>
+        <v>0.955</v>
       </c>
       <c r="J2" t="n">
-        <v>0.179</v>
+        <v>0.173</v>
       </c>
       <c r="K2" t="n">
-        <v>0.859</v>
+        <v>0.839</v>
       </c>
       <c r="L2" t="n">
-        <v>0.286</v>
+        <v>0.308</v>
       </c>
       <c r="M2" t="n">
-        <v>0.837</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>0.29</v>
+        <v>0.312</v>
       </c>
       <c r="O2" t="n">
-        <v>31.6</v>
+        <v>31</v>
       </c>
       <c r="P2" t="n">
-        <v>12.936</v>
+        <v>13.065</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.378</v>
+        <v>1.42</v>
       </c>
       <c r="R2" t="n">
-        <v>0.912</v>
+        <v>0.906</v>
       </c>
     </row>
     <row r="3">
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,7 +994,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P008</t>
+          <t>P007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1004,14 +1004,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>table|comparison|footnote|condition</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D8" t="n">
         <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F8" t="n">
         <v>6</v>
@@ -1023,25 +1023,25 @@
         <v>0.1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P009</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1051,44 +1051,44 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>table|comparison|footnote|condition</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="F9" t="n">
         <v>6</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P010</t>
+          <t>P009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1098,44 +1098,44 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>figure_text|comparison</t>
+          <t>footnote|condition</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="F10" t="n">
         <v>6</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P011</t>
+          <t>P010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1145,20 +1145,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>figure_text|comparison</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F11" t="n">
         <v>6</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H11" t="n">
         <v>0.1</v>
@@ -1170,19 +1170,19 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P012</t>
+          <t>P011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1192,14 +1192,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>table|identifier</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F12" t="n">
         <v>6</v>
@@ -1229,7 +1229,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P013</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1239,17 +1239,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>table|comparison</t>
+          <t>table|identifier</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
@@ -1276,7 +1276,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P014</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1286,17 +1286,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>table|condition|procedure</t>
+          <t>table|comparison</t>
         </is>
       </c>
       <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1323,7 +1323,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P015</t>
+          <t>P014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1333,14 +1333,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>table|condition</t>
+          <t>table|condition|procedure</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F15" t="n">
         <v>6</v>
@@ -1370,7 +1370,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1387,7 +1387,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F16" t="n">
         <v>6</v>
@@ -1417,7 +1417,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P017</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1427,14 +1427,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>table|condition|comparison</t>
+          <t>table|condition</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F17" t="n">
         <v>6</v>
@@ -1464,7 +1464,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P018</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1474,17 +1474,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>table|condition|comparison</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
@@ -1511,7 +1511,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P019</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>causal_relation|condition</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -1549,16 +1549,16 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1568,14 +1568,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>causal_relation|condition</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="F20" t="n">
         <v>8</v>
@@ -1596,16 +1596,16 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P021</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1615,20 +1615,20 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>condition|causal_relation</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>0.1</v>
@@ -1640,7 +1640,7 @@
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -1652,7 +1652,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P022</t>
+          <t>P021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1662,20 +1662,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>procedure|spatial_text</t>
+          <t>condition|causal_relation</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F22" t="n">
         <v>6</v>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H22" t="n">
         <v>0.1</v>
@@ -1687,7 +1687,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -1699,7 +1699,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P023</t>
+          <t>P022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1709,14 +1709,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>condition|causal_relation</t>
+          <t>procedure|spatial_text</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="F23" t="n">
         <v>6</v>
@@ -1725,7 +1725,7 @@
         <v>1</v>
       </c>
       <c r="H23" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -1740,13 +1740,13 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P024</t>
+          <t>P023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1756,14 +1756,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>identifier|condition</t>
+          <t>condition|causal_relation</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F24" t="n">
         <v>6</v>
@@ -1772,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -1787,13 +1787,13 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P025</t>
+          <t>P024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1803,17 +1803,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>footnote|condition|identifier</t>
+          <t>identifier|condition</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="F25" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G25" t="n">
         <v>1</v>
@@ -1840,7 +1840,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P026</t>
+          <t>P025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1850,14 +1850,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>footnote|condition|identifier</t>
         </is>
       </c>
       <c r="D26" t="n">
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="F26" t="n">
         <v>9</v>
@@ -1887,7 +1887,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P027</t>
+          <t>P026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1904,10 +1904,10 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -1934,7 +1934,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P028</t>
+          <t>P027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1944,14 +1944,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>figure_text|identifier</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F28" t="n">
         <v>6</v>
@@ -1981,7 +1981,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P029</t>
+          <t>P028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1991,14 +1991,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>figure_text|identifier</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F29" t="n">
         <v>6</v>
@@ -2007,7 +2007,7 @@
         <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I29" t="n">
         <v>1</v>
@@ -2022,13 +2022,13 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>P030</t>
+          <t>P029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2038,14 +2038,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>comparison|multi_evidence</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="F30" t="n">
         <v>6</v>
@@ -2054,7 +2054,7 @@
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
@@ -2063,19 +2063,19 @@
         <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P031</t>
+          <t>P030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2085,14 +2085,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>comparison|multi_evidence</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="F31" t="n">
         <v>6</v>
@@ -2101,7 +2101,7 @@
         <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -2110,10 +2110,10 @@
         <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
@@ -2122,7 +2122,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P032</t>
+          <t>P031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2132,14 +2132,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F32" t="n">
         <v>6</v>
@@ -2169,7 +2169,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>P033</t>
+          <t>P032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2179,14 +2179,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>footnote|condition|multi_evidence</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="F33" t="n">
         <v>6</v>
@@ -2195,7 +2195,7 @@
         <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
@@ -2204,19 +2204,19 @@
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>P034</t>
+          <t>P033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2226,23 +2226,23 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>comparison|multi_evidence</t>
+          <t>footnote|condition|multi_evidence</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="F34" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I34" t="n">
         <v>1</v>
@@ -2257,13 +2257,13 @@
         <v>0.5</v>
       </c>
       <c r="M34" t="n">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>P035</t>
+          <t>P034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2273,23 +2273,23 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>condition|comparison</t>
+          <t>comparison|multi_evidence</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F35" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G35" t="n">
         <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
@@ -2298,19 +2298,19 @@
         <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>P036</t>
+          <t>P035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2320,14 +2320,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>condition|comparison</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F36" t="n">
         <v>6</v>
@@ -2357,7 +2357,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>P037</t>
+          <t>P036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2367,14 +2367,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>table|footnote|condition</t>
+          <t>table</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F37" t="n">
         <v>6</v>
@@ -2383,7 +2383,7 @@
         <v>1</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I37" t="n">
         <v>1</v>
@@ -2398,13 +2398,13 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P038</t>
+          <t>P037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2414,23 +2414,23 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>table|footnote|condition</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G38" t="n">
         <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I38" t="n">
         <v>1</v>
@@ -2445,13 +2445,13 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>P039</t>
+          <t>P038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2461,29 +2461,29 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="F39" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G39" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
         <v>0.1</v>
       </c>
       <c r="I39" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
         <v>1</v>
@@ -2492,13 +2492,13 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>P040</t>
+          <t>P039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2508,29 +2508,29 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>table|comparison|condition</t>
+          <t>footnote|condition</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F40" t="n">
         <v>6</v>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H40" t="n">
         <v>0.1</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
@@ -2539,13 +2539,13 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P041</t>
+          <t>P040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2555,14 +2555,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>table|comparison|condition</t>
         </is>
       </c>
       <c r="D41" t="n">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F41" t="n">
         <v>6</v>
@@ -2592,7 +2592,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>P042</t>
+          <t>P041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2602,14 +2602,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>footnote|condition</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F42" t="n">
         <v>6</v>
@@ -2639,7 +2639,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>P043</t>
+          <t>P042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2649,14 +2649,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>table|comparison</t>
+          <t>table</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F43" t="n">
         <v>6</v>
@@ -2674,10 +2674,10 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
@@ -2686,7 +2686,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>P044</t>
+          <t>P043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2696,14 +2696,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>table|footnote|condition</t>
+          <t>table|comparison</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F44" t="n">
         <v>6</v>
@@ -2712,7 +2712,7 @@
         <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -2721,19 +2721,19 @@
         <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M44" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>P045</t>
+          <t>P044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2743,23 +2743,23 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>table|footnote|condition</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E45" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F45" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
       </c>
       <c r="H45" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -2768,19 +2768,19 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>P046</t>
+          <t>P045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2790,14 +2790,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>figure_text|footnote</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="F46" t="n">
         <v>9</v>
@@ -2806,19 +2806,19 @@
         <v>1</v>
       </c>
       <c r="H46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="n">
+        <v>5</v>
+      </c>
+      <c r="L46" t="n">
         <v>0.2</v>
-      </c>
-      <c r="I46" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" t="n">
-        <v>1</v>
-      </c>
-      <c r="K46" t="n">
-        <v>2</v>
-      </c>
-      <c r="L46" t="n">
-        <v>1</v>
       </c>
       <c r="M46" t="n">
         <v>1</v>
@@ -2827,33 +2827,33 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>P001</t>
+          <t>P046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>off</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>figure_text|footnote</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="F47" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G47" t="n">
         <v>1</v>
       </c>
       <c r="H47" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
@@ -2865,7 +2865,7 @@
         <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M47" t="n">
         <v>1</v>
@@ -2874,24 +2874,24 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>P002</t>
+          <t>P047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>off</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>table|comparison</t>
         </is>
       </c>
       <c r="D48" t="n">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="F48" t="n">
         <v>6</v>
@@ -2900,7 +2900,7 @@
         <v>1</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="I48" t="n">
         <v>1</v>
@@ -2909,10 +2909,10 @@
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M48" t="n">
         <v>1</v>
@@ -2921,33 +2921,33 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>P003</t>
+          <t>P048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>off</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>table|identifier</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F49" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G49" t="n">
         <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
@@ -2956,104 +2956,104 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>P004</t>
+          <t>P049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>off</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>table|condition</t>
+          <t>multi_document|table|comparison|footnote|condition</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E50" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F50" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="H50" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="K50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>P005</t>
+          <t>P050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>off</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>condition|footnote</t>
+          <t>multi_document|comparison|attribute_leakage</t>
         </is>
       </c>
       <c r="D51" t="n">
         <v>3</v>
       </c>
       <c r="E51" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="F51" t="n">
         <v>6</v>
       </c>
       <c r="G51" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" t="n">
         <v>0.3333333333333333</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" t="n">
-        <v>1</v>
-      </c>
-      <c r="K51" t="n">
-        <v>1</v>
-      </c>
-      <c r="L51" t="n">
-        <v>1</v>
       </c>
       <c r="M51" t="n">
         <v>0.3333333333333333</v>
@@ -3062,7 +3062,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>P006</t>
+          <t>P001</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3072,17 +3072,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>table|comparison|condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D52" t="n">
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F52" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G52" t="n">
         <v>1</v>
@@ -3097,10 +3097,10 @@
         <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M52" t="n">
         <v>1</v>
@@ -3109,7 +3109,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>P008</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3119,44 +3119,44 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>table|comparison|footnote|condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="F53" t="n">
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H53" t="n">
         <v>0.1</v>
       </c>
       <c r="I53" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" t="n">
+        <v>2</v>
+      </c>
+      <c r="L53" t="n">
         <v>0.5</v>
       </c>
-      <c r="J53" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K53" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" t="n">
-        <v>1</v>
-      </c>
       <c r="M53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>P009</t>
+          <t>P003</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3166,44 +3166,44 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D54" t="n">
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F54" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>P010</t>
+          <t>P004</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3213,20 +3213,20 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>figure_text|comparison</t>
+          <t>table|condition</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G55" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H55" t="n">
         <v>0.1</v>
@@ -3241,16 +3241,16 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>P011</t>
+          <t>P005</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3260,20 +3260,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>condition|footnote</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E56" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F56" t="n">
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H56" t="n">
         <v>0.1</v>
@@ -3291,13 +3291,13 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>P012</t>
+          <t>P006</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3307,17 +3307,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>table|identifier</t>
+          <t>table|comparison|condition</t>
         </is>
       </c>
       <c r="D57" t="n">
         <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F57" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G57" t="n">
         <v>1</v>
@@ -3344,7 +3344,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>P013</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3354,29 +3354,29 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>table|comparison</t>
+          <t>table|comparison|footnote|condition</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E58" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F58" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H58" t="n">
         <v>0.1</v>
       </c>
       <c r="I58" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K58" t="n">
         <v>1</v>
@@ -3385,13 +3385,13 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>P014</t>
+          <t>P009</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3401,44 +3401,44 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>table|condition|procedure</t>
+          <t>footnote|condition</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="F59" t="n">
         <v>6</v>
       </c>
       <c r="G59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K59" t="n">
         <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>P015</t>
+          <t>P010</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>table|condition</t>
+          <t>figure_text|comparison</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E60" t="n">
         <v>22</v>
@@ -3461,7 +3461,7 @@
         <v>6</v>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H60" t="n">
         <v>0.1</v>
@@ -3476,16 +3476,16 @@
         <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P011</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3495,14 +3495,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>table|condition</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D61" t="n">
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F61" t="n">
         <v>6</v>
@@ -3532,7 +3532,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>P017</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3542,14 +3542,14 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>table|condition|comparison</t>
+          <t>table|identifier</t>
         </is>
       </c>
       <c r="D62" t="n">
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F62" t="n">
         <v>6</v>
@@ -3579,7 +3579,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>P018</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3589,14 +3589,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>table|comparison</t>
         </is>
       </c>
       <c r="D63" t="n">
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F63" t="n">
         <v>9</v>
@@ -3626,7 +3626,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>P019</t>
+          <t>P014</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3636,17 +3636,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>causal_relation|condition</t>
+          <t>table|condition|procedure</t>
         </is>
       </c>
       <c r="D64" t="n">
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="F64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G64" t="n">
         <v>1</v>
@@ -3664,16 +3664,16 @@
         <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>P015</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3683,17 +3683,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>table|condition</t>
         </is>
       </c>
       <c r="D65" t="n">
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G65" t="n">
         <v>1</v>
@@ -3711,16 +3711,16 @@
         <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>P021</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3730,20 +3730,20 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>condition|causal_relation</t>
+          <t>table|condition</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F66" t="n">
         <v>6</v>
       </c>
       <c r="G66" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H66" t="n">
         <v>0.1</v>
@@ -3755,7 +3755,7 @@
         <v>1</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>1</v>
@@ -3767,7 +3767,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>P022</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3777,14 +3777,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>procedure|spatial_text</t>
+          <t>table|condition|comparison</t>
         </is>
       </c>
       <c r="D67" t="n">
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="F67" t="n">
         <v>6</v>
@@ -3814,7 +3814,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>P023</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3824,23 +3824,23 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>condition|causal_relation</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F68" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G68" t="n">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I68" t="n">
         <v>1</v>
@@ -3849,7 +3849,7 @@
         <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>1</v>
@@ -3861,7 +3861,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>P024</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3871,17 +3871,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>identifier|condition</t>
+          <t>causal_relation|condition</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F69" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G69" t="n">
         <v>1</v>
@@ -3899,16 +3899,16 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>P025</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>footnote|condition|identifier</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3928,7 +3928,7 @@
         <v>48</v>
       </c>
       <c r="F70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G70" t="n">
         <v>1</v>
@@ -3943,19 +3943,19 @@
         <v>1</v>
       </c>
       <c r="K70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="M70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>P026</t>
+          <t>P021</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3965,20 +3965,20 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>condition|causal_relation</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="F71" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H71" t="n">
         <v>0.1</v>
@@ -3990,7 +3990,7 @@
         <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L71" t="n">
         <v>1</v>
@@ -4002,7 +4002,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>P027</t>
+          <t>P022</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4012,14 +4012,14 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>procedure|condition</t>
+          <t>procedure|spatial_text</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="F72" t="n">
         <v>6</v>
@@ -4049,7 +4049,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>P028</t>
+          <t>P023</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4059,14 +4059,14 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>figure_text|identifier</t>
+          <t>condition|causal_relation</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E73" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F73" t="n">
         <v>6</v>
@@ -4075,7 +4075,7 @@
         <v>1</v>
       </c>
       <c r="H73" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I73" t="n">
         <v>1</v>
@@ -4084,7 +4084,7 @@
         <v>1</v>
       </c>
       <c r="K73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L73" t="n">
         <v>1</v>
@@ -4096,7 +4096,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>P029</t>
+          <t>P024</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4106,14 +4106,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>identifier|condition</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F74" t="n">
         <v>6</v>
@@ -4122,7 +4122,7 @@
         <v>1</v>
       </c>
       <c r="H74" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I74" t="n">
         <v>1</v>
@@ -4137,13 +4137,13 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>P030</t>
+          <t>P025</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4153,44 +4153,44 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>comparison|multi_evidence</t>
+          <t>footnote|condition|identifier</t>
         </is>
       </c>
       <c r="D75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" t="n">
+        <v>48</v>
+      </c>
+      <c r="F75" t="n">
+        <v>9</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I75" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" t="n">
         <v>3</v>
       </c>
-      <c r="E75" t="n">
-        <v>38</v>
-      </c>
-      <c r="F75" t="n">
-        <v>6</v>
-      </c>
-      <c r="G75" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I75" t="n">
-        <v>1</v>
-      </c>
-      <c r="J75" t="n">
-        <v>1</v>
-      </c>
-      <c r="K75" t="n">
-        <v>1</v>
-      </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>P031</t>
+          <t>P026</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4200,17 +4200,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D76" t="n">
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F76" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G76" t="n">
         <v>1</v>
@@ -4237,7 +4237,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>P032</t>
+          <t>P027</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4254,7 +4254,7 @@
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F77" t="n">
         <v>6</v>
@@ -4284,7 +4284,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>P033</t>
+          <t>P028</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4294,14 +4294,14 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>footnote|condition|multi_evidence</t>
+          <t>figure_text|identifier</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="F78" t="n">
         <v>6</v>
@@ -4310,7 +4310,7 @@
         <v>1</v>
       </c>
       <c r="H78" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="I78" t="n">
         <v>1</v>
@@ -4319,19 +4319,19 @@
         <v>1</v>
       </c>
       <c r="K78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L78" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>P034</t>
+          <t>P029</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4341,17 +4341,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>comparison|multi_evidence</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>2</v>
       </c>
       <c r="E79" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F79" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G79" t="n">
         <v>1</v>
@@ -4366,10 +4366,10 @@
         <v>1</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M79" t="n">
         <v>0.5</v>
@@ -4378,7 +4378,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>P035</t>
+          <t>P030</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4388,14 +4388,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>condition|comparison</t>
+          <t>comparison|multi_evidence</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E80" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="F80" t="n">
         <v>6</v>
@@ -4404,7 +4404,7 @@
         <v>1</v>
       </c>
       <c r="H80" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I80" t="n">
         <v>1</v>
@@ -4413,19 +4413,19 @@
         <v>1</v>
       </c>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>P036</t>
+          <t>P031</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4435,14 +4435,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F81" t="n">
         <v>6</v>
@@ -4472,7 +4472,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>P037</t>
+          <t>P032</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4482,14 +4482,14 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>table|footnote|condition</t>
+          <t>procedure|condition</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F82" t="n">
         <v>6</v>
@@ -4498,7 +4498,7 @@
         <v>1</v>
       </c>
       <c r="H82" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I82" t="n">
         <v>1</v>
@@ -4513,13 +4513,13 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>P038</t>
+          <t>P033</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4529,23 +4529,23 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>condition|text</t>
+          <t>footnote|condition|multi_evidence</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E83" t="n">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="F83" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G83" t="n">
         <v>1</v>
       </c>
       <c r="H83" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I83" t="n">
         <v>1</v>
@@ -4554,19 +4554,19 @@
         <v>1</v>
       </c>
       <c r="K83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L83" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M83" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>P039</t>
+          <t>P034</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4576,35 +4576,35 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>comparison|multi_evidence</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F84" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I84" t="n">
+        <v>1</v>
+      </c>
+      <c r="J84" t="n">
+        <v>1</v>
+      </c>
+      <c r="K84" t="n">
+        <v>2</v>
+      </c>
+      <c r="L84" t="n">
         <v>0.5</v>
-      </c>
-      <c r="H84" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I84" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J84" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K84" t="n">
-        <v>1</v>
-      </c>
-      <c r="L84" t="n">
-        <v>1</v>
       </c>
       <c r="M84" t="n">
         <v>0.5</v>
@@ -4613,7 +4613,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>P040</t>
+          <t>P035</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4623,14 +4623,14 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>table|comparison|condition</t>
+          <t>condition|comparison</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F85" t="n">
         <v>6</v>
@@ -4648,10 +4648,10 @@
         <v>1</v>
       </c>
       <c r="K85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L85" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M85" t="n">
         <v>1</v>
@@ -4660,7 +4660,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>P041</t>
+          <t>P036</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4670,14 +4670,14 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>footnote|condition</t>
+          <t>table</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F86" t="n">
         <v>6</v>
@@ -4707,7 +4707,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>P042</t>
+          <t>P037</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4717,11 +4717,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>table|footnote|condition</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" t="n">
         <v>20</v>
@@ -4733,7 +4733,7 @@
         <v>1</v>
       </c>
       <c r="H87" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I87" t="n">
         <v>1</v>
@@ -4748,13 +4748,13 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>P043</t>
+          <t>P038</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4764,17 +4764,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>table|comparison</t>
+          <t>condition|text</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="F88" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G88" t="n">
         <v>1</v>
@@ -4789,19 +4789,19 @@
         <v>1</v>
       </c>
       <c r="K88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L88" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>P044</t>
+          <t>P039</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4811,29 +4811,29 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>table|footnote|condition</t>
+          <t>footnote|condition</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>2</v>
       </c>
       <c r="E89" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F89" t="n">
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H89" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J89" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K89" t="n">
         <v>1</v>
@@ -4848,7 +4848,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>P045</t>
+          <t>P040</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4858,17 +4858,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>table|comparison|condition</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="F90" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G90" t="n">
         <v>1</v>
@@ -4883,59 +4883,294 @@
         <v>1</v>
       </c>
       <c r="K90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>P041</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>footnote|condition</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" t="n">
+        <v>30</v>
+      </c>
+      <c r="F91" t="n">
+        <v>6</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I91" t="n">
+        <v>1</v>
+      </c>
+      <c r="J91" t="n">
+        <v>1</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1</v>
+      </c>
+      <c r="L91" t="n">
+        <v>1</v>
+      </c>
+      <c r="M91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>P042</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>20</v>
+      </c>
+      <c r="F92" t="n">
+        <v>6</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I92" t="n">
+        <v>1</v>
+      </c>
+      <c r="J92" t="n">
+        <v>1</v>
+      </c>
+      <c r="K92" t="n">
+        <v>1</v>
+      </c>
+      <c r="L92" t="n">
+        <v>1</v>
+      </c>
+      <c r="M92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>P043</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>table|comparison</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" t="n">
+        <v>23</v>
+      </c>
+      <c r="F93" t="n">
+        <v>6</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I93" t="n">
+        <v>1</v>
+      </c>
+      <c r="J93" t="n">
+        <v>1</v>
+      </c>
+      <c r="K93" t="n">
+        <v>2</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>P044</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>table|footnote|condition</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" t="n">
+        <v>20</v>
+      </c>
+      <c r="F94" t="n">
+        <v>6</v>
+      </c>
+      <c r="G94" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I94" t="n">
+        <v>1</v>
+      </c>
+      <c r="J94" t="n">
+        <v>1</v>
+      </c>
+      <c r="K94" t="n">
+        <v>1</v>
+      </c>
+      <c r="L94" t="n">
+        <v>1</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>P045</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>60</v>
+      </c>
+      <c r="F95" t="n">
+        <v>9</v>
+      </c>
+      <c r="G95" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I95" t="n">
+        <v>1</v>
+      </c>
+      <c r="J95" t="n">
+        <v>1</v>
+      </c>
+      <c r="K95" t="n">
+        <v>2</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>P046</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>on</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>figure_text|footnote</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D96" t="n">
         <v>2</v>
       </c>
-      <c r="E91" t="n">
+      <c r="E96" t="n">
         <v>41</v>
       </c>
-      <c r="F91" t="n">
+      <c r="F96" t="n">
         <v>9</v>
       </c>
-      <c r="G91" t="n">
-        <v>1</v>
-      </c>
-      <c r="H91" t="n">
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" t="n">
         <v>0.2</v>
       </c>
-      <c r="I91" t="n">
-        <v>1</v>
-      </c>
-      <c r="J91" t="n">
-        <v>1</v>
-      </c>
-      <c r="K91" t="n">
+      <c r="I96" t="n">
+        <v>1</v>
+      </c>
+      <c r="J96" t="n">
+        <v>1</v>
+      </c>
+      <c r="K96" t="n">
         <v>2</v>
       </c>
-      <c r="L91" t="n">
+      <c r="L96" t="n">
         <v>0.5</v>
       </c>
-      <c r="M91" t="n">
+      <c r="M96" t="n">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>